<commit_message>
Update dashboard data and site UI for pobreza, ingresos, and empleo.
Refresh Stata processing scripts, move empleo dashboard code to Dashboards/codigo, and regenerate exported Excel datasets.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Dashboards/data/Data final/empleo/empleo adecuado/empleo_demografico.xlsx
+++ b/Dashboards/data/Data final/empleo/empleo adecuado/empleo_demografico.xlsx
@@ -2501,7 +2501,7 @@
         <v>8</v>
       </c>
       <c r="D170" s="1">
-        <v>17.753715515136719</v>
+        <v>20.021692276000977</v>
       </c>
     </row>
     <row r="171">
@@ -2515,7 +2515,7 @@
         <v>9</v>
       </c>
       <c r="D171" s="1">
-        <v>41.799789428710938</v>
+        <v>40.991466522216797</v>
       </c>
     </row>
     <row r="172">
@@ -2529,7 +2529,7 @@
         <v>10</v>
       </c>
       <c r="D172" s="1">
-        <v>27.599956512451172</v>
+        <v>27.007541656494141</v>
       </c>
     </row>
     <row r="173">
@@ -2543,7 +2543,7 @@
         <v>11</v>
       </c>
       <c r="D173" s="1">
-        <v>38.796684265136719</v>
+        <v>39.166553497314453</v>
       </c>
     </row>
     <row r="174">
@@ -2557,7 +2557,7 @@
         <v>12</v>
       </c>
       <c r="D174" s="1">
-        <v>13.119809150695801</v>
+        <v>15.108309745788574</v>
       </c>
     </row>
     <row r="175">
@@ -2571,7 +2571,7 @@
         <v>13</v>
       </c>
       <c r="D175" s="1">
-        <v>27.600553512573242</v>
+        <v>27.681140899658203</v>
       </c>
     </row>
     <row r="176">
@@ -2585,7 +2585,7 @@
         <v>14</v>
       </c>
       <c r="D176" s="1">
-        <v>58.910137176513672</v>
+        <v>61.855678558349609</v>
       </c>
     </row>
     <row r="177">
@@ -2599,7 +2599,7 @@
         <v>15</v>
       </c>
       <c r="D177" s="1">
-        <v>37.895465850830078</v>
+        <v>38.224624633789062</v>
       </c>
     </row>
     <row r="178">
@@ -2613,7 +2613,7 @@
         <v>16</v>
       </c>
       <c r="D178" s="1">
-        <v>12.372861862182617</v>
+        <v>14.166234016418457</v>
       </c>
     </row>
     <row r="179">
@@ -2627,7 +2627,7 @@
         <v>17</v>
       </c>
       <c r="D179" s="1">
-        <v>31.144979476928711</v>
+        <v>30.657489776611328</v>
       </c>
     </row>
     <row r="180">
@@ -2641,7 +2641,7 @@
         <v>18</v>
       </c>
       <c r="D180" s="1">
-        <v>39.128192901611328</v>
+        <v>38.947135925292969</v>
       </c>
     </row>
     <row r="181">
@@ -2655,7 +2655,7 @@
         <v>19</v>
       </c>
       <c r="D181" s="1">
-        <v>26.283281326293945</v>
+        <v>27.201536178588867</v>
       </c>
     </row>
     <row r="182">
@@ -2669,7 +2669,7 @@
         <v>8</v>
       </c>
       <c r="D182" s="1">
-        <v>18.092460632324219</v>
+        <v>19.988697052001953</v>
       </c>
     </row>
     <row r="183">
@@ -2683,7 +2683,7 @@
         <v>9</v>
       </c>
       <c r="D183" s="1">
-        <v>44.401477813720703</v>
+        <v>44.528144836425781</v>
       </c>
     </row>
     <row r="184">
@@ -2697,7 +2697,7 @@
         <v>10</v>
       </c>
       <c r="D184" s="1">
-        <v>28.033050537109375</v>
+        <v>29.717939376831055</v>
       </c>
     </row>
     <row r="185">
@@ -2711,7 +2711,7 @@
         <v>11</v>
       </c>
       <c r="D185" s="1">
-        <v>40.989501953125</v>
+        <v>40.734779357910156</v>
       </c>
     </row>
     <row r="186">
@@ -2725,7 +2725,7 @@
         <v>12</v>
       </c>
       <c r="D186" s="1">
-        <v>15.260344505310059</v>
+        <v>18.204696655273438</v>
       </c>
     </row>
     <row r="187">
@@ -2739,7 +2739,7 @@
         <v>13</v>
       </c>
       <c r="D187" s="1">
-        <v>28.817474365234375</v>
+        <v>29.378194808959961</v>
       </c>
     </row>
     <row r="188">
@@ -2753,7 +2753,7 @@
         <v>14</v>
       </c>
       <c r="D188" s="1">
-        <v>65.214385986328125</v>
+        <v>65.599929809570312</v>
       </c>
     </row>
     <row r="189">
@@ -2767,7 +2767,7 @@
         <v>15</v>
       </c>
       <c r="D189" s="1">
-        <v>40.184112548828125</v>
+        <v>40.767242431640625</v>
       </c>
     </row>
     <row r="190">
@@ -2781,7 +2781,7 @@
         <v>16</v>
       </c>
       <c r="D190" s="1">
-        <v>11.992931365966797</v>
+        <v>13.507410049438477</v>
       </c>
     </row>
     <row r="191">
@@ -2795,7 +2795,7 @@
         <v>17</v>
       </c>
       <c r="D191" s="1">
-        <v>30.73963737487793</v>
+        <v>30.205644607543945</v>
       </c>
     </row>
     <row r="192">
@@ -2809,7 +2809,7 @@
         <v>18</v>
       </c>
       <c r="D192" s="1">
-        <v>40.912242889404297</v>
+        <v>41.124927520751953</v>
       </c>
     </row>
     <row r="193">
@@ -2823,7 +2823,7 @@
         <v>19</v>
       </c>
       <c r="D193" s="1">
-        <v>28.047586441040039</v>
+        <v>28.808261871337891</v>
       </c>
     </row>
     <row r="194">
@@ -2837,7 +2837,7 @@
         <v>8</v>
       </c>
       <c r="D194" s="1">
-        <v>17.974037170410156</v>
+        <v>18.13786506652832</v>
       </c>
     </row>
     <row r="195">
@@ -2851,7 +2851,7 @@
         <v>9</v>
       </c>
       <c r="D195" s="1">
-        <v>45.535945892333984</v>
+        <v>45.274173736572266</v>
       </c>
     </row>
     <row r="196">
@@ -2865,7 +2865,7 @@
         <v>10</v>
       </c>
       <c r="D196" s="1">
-        <v>28.363069534301758</v>
+        <v>27.164226531982422</v>
       </c>
     </row>
     <row r="197">
@@ -2879,7 +2879,7 @@
         <v>11</v>
       </c>
       <c r="D197" s="1">
-        <v>41.946788787841797</v>
+        <v>42.241413116455078</v>
       </c>
     </row>
     <row r="198">
@@ -2893,7 +2893,7 @@
         <v>12</v>
       </c>
       <c r="D198" s="1">
-        <v>15.271793365478516</v>
+        <v>14.002029418945312</v>
       </c>
     </row>
     <row r="199">
@@ -2907,7 +2907,7 @@
         <v>13</v>
       </c>
       <c r="D199" s="1">
-        <v>29.491596221923828</v>
+        <v>29.213476181030273</v>
       </c>
     </row>
     <row r="200">
@@ -2921,7 +2921,7 @@
         <v>14</v>
       </c>
       <c r="D200" s="1">
-        <v>66.002090454101562</v>
+        <v>67.46893310546875</v>
       </c>
     </row>
     <row r="201">
@@ -2935,7 +2935,7 @@
         <v>15</v>
       </c>
       <c r="D201" s="1">
-        <v>41.675064086914062</v>
+        <v>41.139442443847656</v>
       </c>
     </row>
     <row r="202">
@@ -2949,7 +2949,7 @@
         <v>16</v>
       </c>
       <c r="D202" s="1">
-        <v>11.523041725158691</v>
+        <v>13.550883293151855</v>
       </c>
     </row>
     <row r="203">
@@ -2963,7 +2963,7 @@
         <v>17</v>
       </c>
       <c r="D203" s="1">
-        <v>31.8876953125</v>
+        <v>31.827722549438477</v>
       </c>
     </row>
     <row r="204">
@@ -2977,7 +2977,7 @@
         <v>18</v>
       </c>
       <c r="D204" s="1">
-        <v>41.095787048339844</v>
+        <v>41.119102478027344</v>
       </c>
     </row>
     <row r="205">
@@ -2991,7 +2991,7 @@
         <v>19</v>
       </c>
       <c r="D205" s="1">
-        <v>29.023605346679688</v>
+        <v>28.752765655517578</v>
       </c>
     </row>
     <row r="206">
@@ -3005,7 +3005,7 @@
         <v>8</v>
       </c>
       <c r="D206" s="1">
-        <v>17.240484237670898</v>
+        <v>17.721895217895508</v>
       </c>
     </row>
     <row r="207">
@@ -3019,7 +3019,7 @@
         <v>9</v>
       </c>
       <c r="D207" s="1">
-        <v>43.310207366943359</v>
+        <v>41.531345367431641</v>
       </c>
     </row>
     <row r="208">
@@ -3033,7 +3033,7 @@
         <v>10</v>
       </c>
       <c r="D208" s="1">
-        <v>28.400806427001953</v>
+        <v>27.128826141357422</v>
       </c>
     </row>
     <row r="209">
@@ -3047,7 +3047,7 @@
         <v>11</v>
       </c>
       <c r="D209" s="1">
-        <v>38.707950592041016</v>
+        <v>37.793849945068359</v>
       </c>
     </row>
     <row r="210">
@@ -3061,7 +3061,7 @@
         <v>12</v>
       </c>
       <c r="D210" s="1">
-        <v>16.903179168701172</v>
+        <v>15.29649543762207</v>
       </c>
     </row>
     <row r="211">
@@ -3075,7 +3075,7 @@
         <v>13</v>
       </c>
       <c r="D211" s="1">
-        <v>27.830947875976562</v>
+        <v>27.143016815185547</v>
       </c>
     </row>
     <row r="212">
@@ -3089,7 +3089,7 @@
         <v>14</v>
       </c>
       <c r="D212" s="1">
-        <v>64.134437561035156</v>
+        <v>66.099479675292969</v>
       </c>
     </row>
     <row r="213">
@@ -3103,7 +3103,7 @@
         <v>15</v>
       </c>
       <c r="D213" s="1">
-        <v>39.581081390380859</v>
+        <v>38.481132507324219</v>
       </c>
     </row>
     <row r="214">
@@ -3117,7 +3117,7 @@
         <v>16</v>
       </c>
       <c r="D214" s="1">
-        <v>10.579859733581543</v>
+        <v>11.791666030883789</v>
       </c>
     </row>
     <row r="215">
@@ -3131,7 +3131,7 @@
         <v>17</v>
       </c>
       <c r="D215" s="1">
-        <v>29.060214996337891</v>
+        <v>29.267671585083008</v>
       </c>
     </row>
     <row r="216">
@@ -3145,7 +3145,7 @@
         <v>18</v>
       </c>
       <c r="D216" s="1">
-        <v>38.904083251953125</v>
+        <v>37.404815673828125</v>
       </c>
     </row>
     <row r="217">
@@ -3159,7 +3159,7 @@
         <v>19</v>
       </c>
       <c r="D217" s="1">
-        <v>27.345582962036133</v>
+        <v>26.662803649902344</v>
       </c>
     </row>
     <row r="218">
@@ -3173,7 +3173,7 @@
         <v>8</v>
       </c>
       <c r="D218" s="1">
-        <v>18.147819519042969</v>
+        <v>20.154132843017578</v>
       </c>
     </row>
     <row r="219">
@@ -3187,7 +3187,7 @@
         <v>9</v>
       </c>
       <c r="D219" s="1">
-        <v>46.644767761230469</v>
+        <v>46.02447509765625</v>
       </c>
     </row>
     <row r="220">
@@ -3201,7 +3201,7 @@
         <v>10</v>
       </c>
       <c r="D220" s="1">
-        <v>32.413219451904297</v>
+        <v>33.823627471923828</v>
       </c>
     </row>
     <row r="221">
@@ -3215,7 +3215,7 @@
         <v>11</v>
       </c>
       <c r="D221" s="1">
-        <v>41.857810974121094</v>
+        <v>42.099494934082031</v>
       </c>
     </row>
     <row r="222">
@@ -3229,7 +3229,7 @@
         <v>12</v>
       </c>
       <c r="D222" s="1">
-        <v>13.912519454956055</v>
+        <v>13.228731155395508</v>
       </c>
     </row>
     <row r="223">
@@ -3243,7 +3243,7 @@
         <v>13</v>
       </c>
       <c r="D223" s="1">
-        <v>30.809173583984375</v>
+        <v>31.722696304321289</v>
       </c>
     </row>
     <row r="224">
@@ -3257,7 +3257,7 @@
         <v>14</v>
       </c>
       <c r="D224" s="1">
-        <v>65.281341552734375</v>
+        <v>63.745994567871094</v>
       </c>
     </row>
     <row r="225">
@@ -3271,7 +3271,7 @@
         <v>15</v>
       </c>
       <c r="D225" s="1">
-        <v>43.047431945800781</v>
+        <v>42.728805541992188</v>
       </c>
     </row>
     <row r="226">
@@ -3285,7 +3285,7 @@
         <v>16</v>
       </c>
       <c r="D226" s="1">
-        <v>11.55933666229248</v>
+        <v>12.599985122680664</v>
       </c>
     </row>
     <row r="227">
@@ -3299,7 +3299,7 @@
         <v>17</v>
       </c>
       <c r="D227" s="1">
-        <v>33.959747314453125</v>
+        <v>33.715316772460938</v>
       </c>
     </row>
     <row r="228">
@@ -3313,7 +3313,7 @@
         <v>18</v>
       </c>
       <c r="D228" s="1">
-        <v>41.034889221191406</v>
+        <v>41.611598968505859</v>
       </c>
     </row>
     <row r="229">
@@ -3327,7 +3327,7 @@
         <v>19</v>
       </c>
       <c r="D229" s="1">
-        <v>30.626428604125977</v>
+        <v>30.388103485107422</v>
       </c>
     </row>
   </sheetData>

</xml_diff>